<commit_message>
fixed more typos and regenerated reports
</commit_message>
<xml_diff>
--- a/report/risks.xlsx
+++ b/report/risks.xlsx
@@ -19,66 +19,66 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
   <si>
+    <t>Mitigation</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>RAA %</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Likelihood</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
     <t>Technical Asset</t>
   </si>
   <si>
+    <t>Communication Link</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Justification</t>
+  </si>
+  <si>
+    <t>Ticket</t>
+  </si>
+  <si>
+    <t>Risk Category</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Checked by</t>
+  </si>
+  <si>
+    <t>STRIDE</t>
+  </si>
+  <si>
+    <t>CWE</t>
+  </si>
+  <si>
     <t>Identified Risk</t>
   </si>
   <si>
-    <t>Likelihood</t>
-  </si>
-  <si>
-    <t>Impact</t>
-  </si>
-  <si>
-    <t>Risk Category</t>
-  </si>
-  <si>
-    <t>Communication Link</t>
-  </si>
-  <si>
-    <t>RAA %</t>
-  </si>
-  <si>
-    <t>Mitigation</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Ticket</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>Check</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Justification</t>
-  </si>
-  <si>
-    <t>Checked by</t>
-  </si>
-  <si>
-    <t>CWE</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>STRIDE</t>
-  </si>
-  <si>
     <t>Elevated</t>
   </si>
   <si>
@@ -121,7 +121,7 @@
     <t>Are recommendations from the linked cheat sheet and referenced ASVS chapter applied?</t>
   </si>
   <si>
-    <t>missing-authentication@pubic-clients&gt;public-greeting-api-request@pubic-clients@python-http-service</t>
+    <t>missing-authentication@public-clients&gt;public-greeting-api-request@public-clients@python-http-service</t>
   </si>
   <si>
     <t>Unchecked</t>
@@ -178,7 +178,7 @@
     <t>Try to avoid constructing the outgoing target URL with caller controllable values. Alternatively use a mapping (whitelist) when accessing outgoing URLs instead of creating them including caller controllable values. When a third-party product is used instead of custom developed software, check if the product applies the proper mitigation and ensure a reasonable patch-level.</t>
   </si>
   <si>
-    <t>server-side-request-forgery@python-http-service@pubic-clients@python-http-service&gt;public-greeting-api-response</t>
+    <t>server-side-request-forgery@python-http-service@public-clients@python-http-service&gt;public-greeting-api-response</t>
   </si>
   <si>
     <t>CWE-319</t>
@@ -202,13 +202,13 @@
     <t>Apply transport layer encryption to the communication link.</t>
   </si>
   <si>
-    <t>unencrypted-communication@pubic-clients&gt;public-greeting-api-request@pubic-clients@python-http-service</t>
+    <t>unencrypted-communication@public-clients&gt;public-greeting-api-request@public-clients@python-http-service</t>
   </si>
   <si>
     <t>Unencrypted Communication named Public Greeting API Response between Python HTTP Service and Public Clients</t>
   </si>
   <si>
-    <t>unencrypted-communication@python-http-service&gt;public-greeting-api-response@python-http-service@pubic-clients</t>
+    <t>unencrypted-communication@python-http-service&gt;public-greeting-api-response@python-http-service@public-clients</t>
   </si>
   <si>
     <t>Very High</t>
@@ -271,7 +271,7 @@
     <t>Apply an authentication method to the technical asset protecting highly sensitive data via two-factor authentication for human users.</t>
   </si>
   <si>
-    <t>missing-authentication-second-factor@pubic-clients&gt;public-greeting-api-request@pubic-clients@python-http-service</t>
+    <t>missing-authentication-second-factor@public-clients&gt;public-greeting-api-request@public-clients@python-http-service</t>
   </si>
   <si>
     <t>CWE-522</t>
@@ -831,7 +831,7 @@
     <col customWidth="true" max="12" min="12" width="40"/>
     <col customWidth="true" max="13" min="13" width="75"/>
     <col customWidth="true" max="14" min="14" width="66.42857142857143"/>
-    <col customWidth="true" max="15" min="15" width="86.42857142857143"/>
+    <col customWidth="true" max="15" min="15" width="87.85714285714286"/>
     <col customWidth="true" max="16" min="16" width="14.428571428571429"/>
     <col customWidth="true" max="17" min="17" width="20"/>
     <col customWidth="true" max="18" min="18" width="11"/>
@@ -841,64 +841,64 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C1" s="24" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="H1" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="K1" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="L1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="M1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="N1" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="P1" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="R1" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="S1" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="H1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="I1" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="J1" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="K1" s="24" t="s">
-        <v>1</v>
-      </c>
-      <c r="L1" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="N1" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="P1" s="24" t="s">
+      <c r="T1" s="24" t="s">
         <v>13</v>
-      </c>
-      <c r="Q1" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="R1" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="S1" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="T1" s="24" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
initial commit for the risk mitigation tutorial
</commit_message>
<xml_diff>
--- a/report/risks.xlsx
+++ b/report/risks.xlsx
@@ -17,68 +17,68 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+  <si>
+    <t>Risk Category</t>
+  </si>
+  <si>
+    <t>Identified Risk</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Ticket</t>
+  </si>
+  <si>
+    <t>Justification</t>
+  </si>
+  <si>
+    <t>STRIDE</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Technical Asset</t>
+  </si>
+  <si>
+    <t>Communication Link</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
   <si>
     <t>Mitigation</t>
   </si>
   <si>
+    <t>Check</t>
+  </si>
+  <si>
     <t>ID</t>
   </si>
   <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Impact</t>
+    <t>Likelihood</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>CWE</t>
   </si>
   <si>
     <t>RAA %</t>
   </si>
   <si>
-    <t>Check</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Likelihood</t>
-  </si>
-  <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>Technical Asset</t>
-  </si>
-  <si>
-    <t>Communication Link</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>Justification</t>
-  </si>
-  <si>
-    <t>Ticket</t>
-  </si>
-  <si>
-    <t>Risk Category</t>
-  </si>
-  <si>
     <t>Status</t>
   </si>
   <si>
     <t>Checked by</t>
   </si>
   <si>
-    <t>STRIDE</t>
-  </si>
-  <si>
-    <t>CWE</t>
-  </si>
-  <si>
-    <t>Identified Risk</t>
-  </si>
-  <si>
     <t>Elevated</t>
   </si>
   <si>
@@ -124,36 +124,52 @@
     <t>missing-authentication@public-clients&gt;public-greeting-api-request@public-clients@python-http-service</t>
   </si>
   <si>
+    <t>Accepted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">This is a public API that is meant to be accessed by anyone, so we accept the risk of missing authentication.
+</t>
+  </si>
+  <si>
+    <t>2026-01-02</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>Tampering</t>
+  </si>
+  <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>CWE-16</t>
+  </si>
+  <si>
+    <t>Missing Hardening</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Missing Hardening risk at Python HTTP Service</t>
+  </si>
+  <si>
+    <t>System Hardening</t>
+  </si>
+  <si>
+    <t>Try to apply all hardening best practices (like CIS benchmarks, OWASP recommendations, vendor recommendations, DevSec Hardening Framework, DBSAT for Oracle databases, and others).</t>
+  </si>
+  <si>
+    <t>missing-hardening@python-http-service</t>
+  </si>
+  <si>
     <t>Unchecked</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Tampering</t>
-  </si>
-  <si>
-    <t>Operations</t>
-  </si>
-  <si>
-    <t>CWE-16</t>
-  </si>
-  <si>
-    <t>Missing Hardening</t>
-  </si>
-  <si>
-    <t>Missing Hardening risk at Python HTTP Service</t>
-  </si>
-  <si>
-    <t>System Hardening</t>
-  </si>
-  <si>
-    <t>Try to apply all hardening best practices (like CIS benchmarks, OWASP recommendations, vendor recommendations, DevSec Hardening Framework, DBSAT for Oracle databases, and others).</t>
-  </si>
-  <si>
-    <t>missing-hardening@python-http-service</t>
-  </si>
-  <si>
     <t>Information Disclosure</t>
   </si>
   <si>
@@ -211,6 +227,97 @@
     <t>unencrypted-communication@python-http-service&gt;public-greeting-api-response@python-http-service@public-clients</t>
   </si>
   <si>
+    <t>Unlikely</t>
+  </si>
+  <si>
+    <t>CWE-1127</t>
+  </si>
+  <si>
+    <t>Missing Build Infrastructure</t>
+  </si>
+  <si>
+    <t>Missing Build Infrastructure in the threat model (referencing asset Python HTTP Service as an example)</t>
+  </si>
+  <si>
+    <t>Build Pipeline Hardening</t>
+  </si>
+  <si>
+    <t>Include the build infrastructure in the model.</t>
+  </si>
+  <si>
+    <t>missing-build-infrastructure@python-http-service</t>
+  </si>
+  <si>
+    <t>CWE-522</t>
+  </si>
+  <si>
+    <t>Missing Vault (Secret Storage)</t>
+  </si>
+  <si>
+    <t>Missing Vault (Secret Storage) in the threat model (referencing asset Python HTTP Service as an example)</t>
+  </si>
+  <si>
+    <t>Vault (Secret Storage)</t>
+  </si>
+  <si>
+    <t>Consider using a Vault (Secret Storage) to securely store and access config secrets (like credentials, private keys, client certificates, etc.).</t>
+  </si>
+  <si>
+    <t>Is there a Vault (Secret Storage) in place?</t>
+  </si>
+  <si>
+    <t>missing-vault@python-http-service</t>
+  </si>
+  <si>
+    <t>CWE-1008</t>
+  </si>
+  <si>
+    <t>Missing Web Application Firewall (WAF)</t>
+  </si>
+  <si>
+    <t>Missing Web Application Firewall (WAF) risk at Python HTTP Service</t>
+  </si>
+  <si>
+    <t>Web Application Firewall (WAF)</t>
+  </si>
+  <si>
+    <t>Consider placing a Web Application Firewall (WAF) in front of the web-services and/or web-applications. For cloud environments many cloud providers offer pre-configured WAFs. Even reverse proxies can be enhances by a WAF component via ModSecurity plugins.</t>
+  </si>
+  <si>
+    <t>Is there a Web Application Firewall (WAF) in place?</t>
+  </si>
+  <si>
+    <t>missing-waf@python-http-service</t>
+  </si>
+  <si>
+    <t>Business Side</t>
+  </si>
+  <si>
+    <t>CWE-308</t>
+  </si>
+  <si>
+    <t>Missing Two-Factor Authentication (2FA)</t>
+  </si>
+  <si>
+    <t>Missing Two-Factor Authentication covering communication link Public Greeting API Request from Public Clients to Python HTTP Service</t>
+  </si>
+  <si>
+    <t>Authentication with Second Factor (2FA)</t>
+  </si>
+  <si>
+    <t>Apply an authentication method to the technical asset protecting highly sensitive data via two-factor authentication for human users.</t>
+  </si>
+  <si>
+    <t>missing-authentication-second-factor@public-clients&gt;public-greeting-api-request@public-clients@python-http-service</t>
+  </si>
+  <si>
+    <t>Mitigated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">We don't allow authentication at all, so no MFA is required.
+</t>
+  </si>
+  <si>
     <t>Very High</t>
   </si>
   <si>
@@ -232,88 +339,8 @@
     <t>untrusted-deserialization@python-http-service</t>
   </si>
   <si>
-    <t>Unlikely</t>
-  </si>
-  <si>
-    <t>CWE-1127</t>
-  </si>
-  <si>
-    <t>Missing Build Infrastructure</t>
-  </si>
-  <si>
-    <t>Missing Build Infrastructure in the threat model (referencing asset Python HTTP Service as an example)</t>
-  </si>
-  <si>
-    <t>Build Pipeline Hardening</t>
-  </si>
-  <si>
-    <t>Include the build infrastructure in the model.</t>
-  </si>
-  <si>
-    <t>missing-build-infrastructure@python-http-service</t>
-  </si>
-  <si>
-    <t>Business Side</t>
-  </si>
-  <si>
-    <t>CWE-308</t>
-  </si>
-  <si>
-    <t>Missing Two-Factor Authentication (2FA)</t>
-  </si>
-  <si>
-    <t>Missing Two-Factor Authentication covering communication link Public Greeting API Request from Public Clients to Python HTTP Service</t>
-  </si>
-  <si>
-    <t>Authentication with Second Factor (2FA)</t>
-  </si>
-  <si>
-    <t>Apply an authentication method to the technical asset protecting highly sensitive data via two-factor authentication for human users.</t>
-  </si>
-  <si>
-    <t>missing-authentication-second-factor@public-clients&gt;public-greeting-api-request@public-clients@python-http-service</t>
-  </si>
-  <si>
-    <t>CWE-522</t>
-  </si>
-  <si>
-    <t>Missing Vault (Secret Storage)</t>
-  </si>
-  <si>
-    <t>Missing Vault (Secret Storage) in the threat model (referencing asset Python HTTP Service as an example)</t>
-  </si>
-  <si>
-    <t>Vault (Secret Storage)</t>
-  </si>
-  <si>
-    <t>Consider using a Vault (Secret Storage) to securely store and access config secrets (like credentials, private keys, client certificates, etc.).</t>
-  </si>
-  <si>
-    <t>Is there a Vault (Secret Storage) in place?</t>
-  </si>
-  <si>
-    <t>missing-vault@python-http-service</t>
-  </si>
-  <si>
-    <t>CWE-1008</t>
-  </si>
-  <si>
-    <t>Missing Web Application Firewall (WAF)</t>
-  </si>
-  <si>
-    <t>Missing Web Application Firewall (WAF) risk at Python HTTP Service</t>
-  </si>
-  <si>
-    <t>Web Application Firewall (WAF)</t>
-  </si>
-  <si>
-    <t>Consider placing a Web Application Firewall (WAF) in front of the web-services and/or web-applications. For cloud environments many cloud providers offer pre-configured WAFs. Even reverse proxies can be enhances by a WAF component via ModSecurity plugins.</t>
-  </si>
-  <si>
-    <t>Is there a Web Application Firewall (WAF) in place?</t>
-  </si>
-  <si>
-    <t>missing-waf@python-http-service</t>
+    <t xml:space="preserve">The API endpoint will use a safe deserialization library that prevents code execution and other attacks.
+</t>
   </si>
 </sst>
 </file>
@@ -833,72 +860,72 @@
     <col customWidth="true" max="14" min="14" width="66.42857142857143"/>
     <col customWidth="true" max="15" min="15" width="87.85714285714286"/>
     <col customWidth="true" max="16" min="16" width="14.428571428571429"/>
-    <col customWidth="true" max="17" min="17" width="20"/>
-    <col customWidth="true" max="18" min="18" width="11"/>
+    <col customWidth="true" max="17" min="17" width="85"/>
+    <col customWidth="true" max="18" min="18" width="15.285714285714285"/>
     <col customWidth="true" max="19" min="19" width="17"/>
     <col customWidth="true" max="20" min="20" width="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="H1" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="L1" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="M1" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="N1" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="O1" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="P1" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q1" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="R1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1" s="24" t="s">
+      <c r="S1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="T1" s="24" t="s">
         <v>3</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="G1" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="I1" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="J1" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="K1" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="L1" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="N1" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="O1" s="24" t="s">
-        <v>1</v>
-      </c>
-      <c r="P1" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q1" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="R1" s="24" t="s">
-        <v>6</v>
-      </c>
-      <c r="S1" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="T1" s="24" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2">
@@ -947,20 +974,20 @@
       <c r="O2" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="P2" s="13" t="s">
         <v>35</v>
       </c>
       <c r="Q2" s="19" t="s">
         <v>36</v>
       </c>
       <c r="R2" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S2" s="17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="T2" s="16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3">
@@ -974,55 +1001,55 @@
         <v>22</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H3" s="5" t="s">
         <v>27</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J3" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K3" s="19" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="L3" s="23" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="M3" s="23" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N3" s="23" t="s">
         <v>33</v>
       </c>
       <c r="O3" s="20" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="P3" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R3" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S3" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T3" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4">
@@ -1036,55 +1063,55 @@
         <v>22</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>27</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="J4" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="L4" s="23" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="M4" s="23" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="N4" s="23" t="s">
         <v>33</v>
       </c>
       <c r="O4" s="20" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S4" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5">
@@ -1098,55 +1125,55 @@
         <v>22</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="J5" s="18" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="K5" s="19" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="L5" s="23" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="N5" s="23" t="s">
         <v>33</v>
       </c>
       <c r="O5" s="20" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R5" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S5" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T5" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6">
@@ -1160,117 +1187,117 @@
         <v>22</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H6" s="5" t="s">
         <v>27</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="J6" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="L6" s="23" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="M6" s="23" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="N6" s="23" t="s">
         <v>33</v>
       </c>
       <c r="O6" s="20" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R6" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S6" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T6" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>64</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="6" t="s">
+      <c r="A7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="H7" s="5" t="s">
+      <c r="F7" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="I7" s="5" t="s">
-        <v>36</v>
+      <c r="I7" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="J7" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L7" s="23" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="M7" s="23" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="N7" s="23" t="s">
         <v>33</v>
       </c>
       <c r="O7" s="20" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R7" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S7" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T7" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8">
@@ -1278,61 +1305,61 @@
         <v>22</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C8" s="8" t="s">
         <v>22</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>24</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>27</v>
       </c>
       <c r="I8" s="7" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J8" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K8" s="19" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="L8" s="23" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="M8" s="23" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="N8" s="23" t="s">
-        <v>33</v>
+        <v>81</v>
       </c>
       <c r="O8" s="20" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q8" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R8" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S8" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T8" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9">
@@ -1340,185 +1367,185 @@
         <v>22</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C9" s="8" t="s">
         <v>22</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>27</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>28</v>
+        <v>44</v>
       </c>
       <c r="J9" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="L9" s="23" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="M9" s="23" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="N9" s="23" t="s">
-        <v>33</v>
+        <v>88</v>
       </c>
       <c r="O9" s="20" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>35</v>
+        <v>49</v>
       </c>
       <c r="Q9" s="19" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="R9" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="S9" s="17" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="T9" s="16" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C10" s="8" t="s">
+      <c r="B10" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>85</v>
-      </c>
-      <c r="G10" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="H10" s="7" t="s">
+      <c r="D10" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>91</v>
+      </c>
+      <c r="G10" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="H10" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>36</v>
+      <c r="I10" s="21" t="s">
+        <v>28</v>
       </c>
       <c r="J10" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="L10" s="23" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="M10" s="23" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="N10" s="23" t="s">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="O10" s="20" t="s">
-        <v>91</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>35</v>
+        <v>96</v>
+      </c>
+      <c r="P10" s="11" t="s">
+        <v>97</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>36</v>
+        <v>98</v>
       </c>
       <c r="R10" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S10" s="17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="T10" s="16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E11" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="G11" s="7" t="s">
-        <v>93</v>
-      </c>
-      <c r="H11" s="7" t="s">
+      <c r="A11" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="G11" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="H11" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="I11" s="7" t="s">
-        <v>36</v>
+      <c r="I11" s="21" t="s">
+        <v>44</v>
       </c>
       <c r="J11" s="18" t="s">
         <v>29</v>
       </c>
       <c r="K11" s="19" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="L11" s="23" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="M11" s="23" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="N11" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="O11" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="P11" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="O11" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="P11" s="10" t="s">
-        <v>35</v>
-      </c>
       <c r="Q11" s="19" t="s">
-        <v>36</v>
+        <v>106</v>
       </c>
       <c r="R11" s="17" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="S11" s="17" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="T11" s="16" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Initial pass for branch.
</commit_message>
<xml_diff>
--- a/report/risks.xlsx
+++ b/report/risks.xlsx
@@ -19,64 +19,64 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
   <si>
+    <t>Function</t>
+  </si>
+  <si>
     <t>Risk Category</t>
   </si>
   <si>
+    <t>RAA %</t>
+  </si>
+  <si>
     <t>Identified Risk</t>
   </si>
   <si>
+    <t>Mitigation</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
     <t>Date</t>
   </si>
   <si>
+    <t>CWE</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>STRIDE</t>
+  </si>
+  <si>
+    <t>Likelihood</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Technical Asset</t>
+  </si>
+  <si>
+    <t>Communication Link</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Checked by</t>
+  </si>
+  <si>
     <t>Ticket</t>
   </si>
   <si>
     <t>Justification</t>
   </si>
   <si>
-    <t>STRIDE</t>
-  </si>
-  <si>
     <t>Severity</t>
-  </si>
-  <si>
-    <t>Impact</t>
-  </si>
-  <si>
-    <t>Technical Asset</t>
-  </si>
-  <si>
-    <t>Communication Link</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>Mitigation</t>
-  </si>
-  <si>
-    <t>Check</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Likelihood</t>
-  </si>
-  <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>CWE</t>
-  </si>
-  <si>
-    <t>RAA %</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Checked by</t>
   </si>
   <si>
     <t>Elevated</t>
@@ -868,64 +868,64 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>14</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="N1" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="O1" s="24" t="s">
+        <v>8</v>
+      </c>
+      <c r="P1" s="24" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q1" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="R1" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B1" s="24" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="24" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="24" t="s">
+      <c r="S1" s="24" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="24" t="s">
-        <v>8</v>
-      </c>
-      <c r="I1" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="J1" s="24" t="s">
+      <c r="T1" s="24" t="s">
         <v>17</v>
-      </c>
-      <c r="K1" s="24" t="s">
-        <v>1</v>
-      </c>
-      <c r="L1" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="24" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q1" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="R1" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="S1" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="T1" s="24" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2">

</xml_diff>

<commit_message>
After reviewing the agenda and how used by code, removing the custom section to be used in a later branch
</commit_message>
<xml_diff>
--- a/report/risks.xlsx
+++ b/report/risks.xlsx
@@ -10,14 +10,59 @@
     <sheet name="Greeting Application" sheetId="2" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'Greeting Application'!$A$1:$T$11</definedName>
+    <definedName hidden="true" localSheetId="0" name="_xlnm._FilterDatabase">'Greeting Application'!$A$1:$T$12</definedName>
   </definedNames>
   <calcPr calcId="122211"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
+  <si>
+    <t>Communication Link</t>
+  </si>
+  <si>
+    <t>RAA %</t>
+  </si>
+  <si>
+    <t>Action</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Impact</t>
+  </si>
+  <si>
+    <t>Function</t>
+  </si>
+  <si>
+    <t>CWE</t>
+  </si>
+  <si>
+    <t>Mitigation</t>
+  </si>
+  <si>
+    <t>Justification</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>Severity</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>STRIDE</t>
+  </si>
+  <si>
+    <t>Likelihood</t>
+  </si>
   <si>
     <t>Risk Category</t>
   </si>
@@ -25,88 +70,79 @@
     <t>Identified Risk</t>
   </si>
   <si>
-    <t>Date</t>
+    <t>Checked by</t>
   </si>
   <si>
     <t>Ticket</t>
   </si>
   <si>
-    <t>Justification</t>
-  </si>
-  <si>
-    <t>STRIDE</t>
-  </si>
-  <si>
-    <t>Severity</t>
-  </si>
-  <si>
-    <t>Impact</t>
-  </si>
-  <si>
     <t>Technical Asset</t>
   </si>
   <si>
-    <t>Communication Link</t>
-  </si>
-  <si>
-    <t>Action</t>
-  </si>
-  <si>
-    <t>Mitigation</t>
-  </si>
-  <si>
-    <t>Check</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>Likelihood</t>
-  </si>
-  <si>
-    <t>Function</t>
-  </si>
-  <si>
-    <t>CWE</t>
-  </si>
-  <si>
-    <t>RAA %</t>
-  </si>
-  <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>Checked by</t>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Likely</t>
+  </si>
+  <si>
+    <t>Denial of Service</t>
+  </si>
+  <si>
+    <t>Architecture</t>
+  </si>
+  <si>
+    <t>CWE-400</t>
+  </si>
+  <si>
+    <t>Unbounded Search Query Cost</t>
+  </si>
+  <si>
+    <t>Python HTTP Service</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>100</t>
+  </si>
+  <si>
+    <t>Unbounded Search Query Cost at Python HTTP Service</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add server-side query limits, pagination limits, timeouts, and rate limits before exposing the search endpoint to public clients.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enforce maximum result sizes and query complexity, apply rate limiting, and monitor for abnormal request patterns.
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test large pagination values, repeated requests, and expensive search combinations while monitoring resource use.
+</t>
+  </si>
+  <si>
+    <t>unbounded-search-query-cost@python-http-service@public-internet</t>
+  </si>
+  <si>
+    <t>Unchecked</t>
   </si>
   <si>
     <t>Elevated</t>
   </si>
   <si>
-    <t>Likely</t>
-  </si>
-  <si>
     <t>Medium</t>
   </si>
   <si>
     <t>Elevation of Privilege</t>
   </si>
   <si>
-    <t>Architecture</t>
-  </si>
-  <si>
     <t>CWE-306</t>
   </si>
   <si>
     <t>Missing Authentication</t>
   </si>
   <si>
-    <t>Python HTTP Service</t>
-  </si>
-  <si>
     <t>Public Greeting API Request</t>
-  </si>
-  <si>
-    <t>100</t>
   </si>
   <si>
     <t>Missing Authentication covering communication link Public Greeting API Request from Public Clients to Python HTTP Service</t>
@@ -152,9 +188,6 @@
     <t>Missing Hardening</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Missing Hardening risk at Python HTTP Service</t>
   </si>
   <si>
@@ -165,9 +198,6 @@
   </si>
   <si>
     <t>missing-hardening@python-http-service</t>
-  </si>
-  <si>
-    <t>Unchecked</t>
   </si>
   <si>
     <t>Information Disclosure</t>
@@ -855,10 +885,9 @@
     <col customWidth="true" max="9" min="9" width="30.71428571428571"/>
     <col customWidth="true" max="10" min="10" width="12"/>
     <col customWidth="true" max="11" min="11" width="75"/>
-    <col customWidth="true" max="12" min="12" width="40"/>
+    <col customWidth="true" max="12" min="12" width="99.28571428571429"/>
     <col customWidth="true" max="13" min="13" width="75"/>
-    <col customWidth="true" max="14" min="14" width="66.42857142857143"/>
-    <col customWidth="true" max="15" min="15" width="87.85714285714286"/>
+    <col customWidth="true" max="15" min="14" width="87.85714285714286"/>
     <col customWidth="true" max="16" min="16" width="14.428571428571429"/>
     <col customWidth="true" max="17" min="17" width="85"/>
     <col customWidth="true" max="18" min="18" width="15.285714285714285"/>
@@ -868,220 +897,220 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B1" s="24" t="s">
         <v>14</v>
       </c>
       <c r="C1" s="24" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="24" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="24" t="s">
+        <v>5</v>
+      </c>
+      <c r="F1" s="24" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="24" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="J1" s="24" t="s">
+        <v>1</v>
+      </c>
+      <c r="K1" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="24" t="s">
+        <v>2</v>
+      </c>
+      <c r="M1" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="24" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="24" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="24" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="24" t="s">
-        <v>0</v>
-      </c>
-      <c r="H1" s="24" t="s">
+      <c r="N1" s="24" t="s">
+        <v>11</v>
+      </c>
+      <c r="O1" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="P1" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="Q1" s="24" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="R1" s="24" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="S1" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="K1" s="24" t="s">
-        <v>1</v>
-      </c>
-      <c r="L1" s="24" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="24" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="24" t="s">
+      <c r="T1" s="24" t="s">
         <v>18</v>
-      </c>
-      <c r="Q1" s="24" t="s">
-        <v>4</v>
-      </c>
-      <c r="R1" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="S1" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="T1" s="24" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J2" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="K2" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="K2" s="19" t="s">
+      <c r="L2" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="23" t="s">
+      <c r="M2" s="23" t="s">
         <v>31</v>
       </c>
-      <c r="M2" s="23" t="s">
+      <c r="N2" s="23" t="s">
         <v>32</v>
       </c>
-      <c r="N2" s="23" t="s">
+      <c r="O2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="O2" s="20" t="s">
+      <c r="P2" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="P2" s="13" t="s">
-        <v>35</v>
-      </c>
       <c r="Q2" s="19" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="R2" s="17" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="S2" s="17" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="T2" s="16" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D3" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I3" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="J3" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="K3" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="L3" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="M3" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="H3" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I3" s="5" t="s">
+      <c r="N3" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="J3" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="K3" s="19" t="s">
+      <c r="O3" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="L3" s="23" t="s">
+      <c r="P3" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="M3" s="23" t="s">
+      <c r="Q3" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="N3" s="23" t="s">
-        <v>33</v>
-      </c>
-      <c r="O3" s="20" t="s">
+      <c r="R3" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="P3" s="10" t="s">
+      <c r="S3" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="Q3" s="19" t="s">
-        <v>44</v>
-      </c>
-      <c r="R3" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="S3" s="17" t="s">
-        <v>44</v>
-      </c>
       <c r="T3" s="16" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>54</v>
+        <v>27</v>
       </c>
       <c r="J4" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K4" s="19" t="s">
         <v>55</v>
@@ -1093,184 +1122,184 @@
         <v>57</v>
       </c>
       <c r="N4" s="23" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="O4" s="20" t="s">
         <v>58</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="R4" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="S4" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="T4" s="16" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="I5" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="J5" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="J5" s="18" t="s">
-        <v>62</v>
-      </c>
       <c r="K5" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="L5" s="23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="M5" s="23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="N5" s="23" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="O5" s="20" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P5" s="10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="R5" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="S5" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="T5" s="16" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="I6" s="5" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="J6" s="18" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="K6" s="19" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L6" s="23" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="M6" s="23" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
       <c r="N6" s="23" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="O6" s="20" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="P6" s="10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="R6" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="S6" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="T6" s="16" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="8" t="s">
+      <c r="A7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I7" s="7" t="s">
-        <v>44</v>
+      <c r="H7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>63</v>
       </c>
       <c r="J7" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K7" s="19" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="L7" s="23" t="s">
         <v>73</v>
@@ -1279,228 +1308,228 @@
         <v>74</v>
       </c>
       <c r="N7" s="23" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="O7" s="20" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="P7" s="10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="R7" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="S7" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="T7" s="16" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I8" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J8" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="L8" s="23" t="s">
+        <v>82</v>
+      </c>
+      <c r="M8" s="23" t="s">
+        <v>83</v>
+      </c>
+      <c r="N8" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="J8" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="K8" s="19" t="s">
-        <v>78</v>
-      </c>
-      <c r="L8" s="23" t="s">
-        <v>79</v>
-      </c>
-      <c r="M8" s="23" t="s">
-        <v>80</v>
-      </c>
-      <c r="N8" s="23" t="s">
-        <v>81</v>
-      </c>
       <c r="O8" s="20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="P8" s="10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="Q8" s="19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="R8" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="S8" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="T8" s="16" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I9" s="7" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="J9" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K9" s="19" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="L9" s="23" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="M9" s="23" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="N9" s="23" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="O9" s="20" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="P9" s="10" t="s">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="Q9" s="19" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="R9" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="S9" s="17" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="T9" s="16" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="17" t="s">
-        <v>69</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="17" t="s">
-        <v>23</v>
-      </c>
-      <c r="E10" s="17" t="s">
-        <v>90</v>
-      </c>
-      <c r="F10" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="G10" s="21" t="s">
+      <c r="A10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="H10" s="21" t="s">
-        <v>27</v>
-      </c>
-      <c r="I10" s="21" t="s">
+      <c r="G10" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="H10" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="J10" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="J10" s="18" t="s">
-        <v>29</v>
-      </c>
       <c r="K10" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="L10" s="23" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M10" s="23" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="N10" s="23" t="s">
-        <v>33</v>
+        <v>97</v>
       </c>
       <c r="O10" s="20" t="s">
-        <v>96</v>
-      </c>
-      <c r="P10" s="11" t="s">
-        <v>97</v>
+        <v>98</v>
+      </c>
+      <c r="P10" s="10" t="s">
+        <v>34</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>98</v>
+        <v>27</v>
       </c>
       <c r="R10" s="17" t="s">
-        <v>37</v>
+        <v>27</v>
       </c>
       <c r="S10" s="17" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="T10" s="16" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="s">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="C11" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="E11" s="17" t="s">
         <v>99</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>24</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>100</v>
@@ -1509,13 +1538,13 @@
         <v>101</v>
       </c>
       <c r="H11" s="21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="I11" s="21" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="J11" s="18" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="K11" s="19" t="s">
         <v>102</v>
@@ -1527,29 +1556,91 @@
         <v>104</v>
       </c>
       <c r="N11" s="23" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="O11" s="20" t="s">
         <v>105</v>
       </c>
       <c r="P11" s="11" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="Q11" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="R11" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="S11" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="T11" s="16" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="G12" s="21" t="s">
+        <v>110</v>
+      </c>
+      <c r="H12" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="I12" s="21" t="s">
+        <v>27</v>
+      </c>
+      <c r="J12" s="18" t="s">
+        <v>28</v>
+      </c>
+      <c r="K12" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>112</v>
+      </c>
+      <c r="M12" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="N12" s="23" t="s">
+        <v>44</v>
+      </c>
+      <c r="O12" s="20" t="s">
+        <v>114</v>
+      </c>
+      <c r="P12" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="R11" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="S11" s="17" t="s">
-        <v>38</v>
-      </c>
-      <c r="T11" s="16" t="s">
-        <v>39</v>
+      <c r="Q12" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="R12" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="S12" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="T12" s="16" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="$A$1:$T$11"/>
+  <autoFilter ref="$A$1:$T$12"/>
   <pageSetup orientation="landscape" paperSize="9"/>
   <headerFooter>
     <oddHeader>&amp;R&amp;P</oddHeader>

</xml_diff>